<commit_message>
Add industrial conversion screens to market memos
</commit_message>
<xml_diff>
--- a/outputs/flowery-branch-i985-industrial-intelligence/Flowery_Branch_I985_Industrial_Entitlement_Landscape.xlsx
+++ b/outputs/flowery-branch-i985-industrial-intelligence/Flowery_Branch_I985_Industrial_Entitlement_Landscape.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rf10597175f2e4051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recent Cases" sheetId="2" r:id="Rfa699a641e624827"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Matrix" sheetId="3" r:id="R0804768203344299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Players" sheetId="4" r:id="R30f4b3e72ba3494f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="5" r:id="R93de3d1b877f40af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Ra753d59cab6b40f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recent Cases" sheetId="2" r:id="R173d9e153e48470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Matrix" sheetId="3" r:id="R912baa7aaee843f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conversion Matrix" sheetId="4" r:id="R76707c2525f24942"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Players" sheetId="5" r:id="Rd67ea4f60ac749e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="6" r:id="R835c6ad100fa410d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -446,7 +447,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>Hardened public-record update | Research window 2021-August 27, 2026 | No open-record requests used</x:v>
+        <x:v>Broker/client handout | Research window 2021-August 27, 2026 | City-limit industrial conversion screen</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -458,7 +459,7 @@
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="24" t="str">
-        <x:v>Investment read: the best I-985 acquisition lane remains existing industrial fabric tied to Falcon Parkway, Thurmon Tanner Parkway, Atlanta Highway, and Exit 12/14. The public packet archive now verifies several local approvals, but the residual diligence line is clear: parcel-to-building crosswalks, permit/CO copies, utility commitments, and non-Flowery jurisdiction files still need direct source pulls.</x:v>
+        <x:v>Broker read: inside Flowery Branch city limits, the cleanest industrial targets are existing M-1 parcels and HB/commercial frontage already aligned with Industrial Employment at I-985 / Thurmon Tanner / Atlanta Highway. Agricultural land can convert to M-1 only when it expands a proven industrial corridor and solves infrastructure. M-2 and quarry-style heavy industry are special-use plays, not ordinary warehouse comps.</x:v>
       </x:c>
       <x:c r="B4" s="25"/>
       <x:c r="C4" s="25"/>
@@ -490,68 +491,68 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="34" t="str">
-        <x:v>Closed / strengthened</x:v>
+        <x:v>Green / Yellow Targets</x:v>
       </x:c>
       <x:c r="B8" s="34" t="str">
-        <x:v>Still open</x:v>
+        <x:v>Orange / Red Targets</x:v>
       </x:c>
       <x:c r="C8" s="34" t="str">
-        <x:v>Why it matters</x:v>
+        <x:v>Customer Rule</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="56" customHeight="1">
       <x:c r="A9" s="37" t="str">
-        <x:v>Project Falcon</x:v>
+        <x:v>Existing M-1 on Atlanta Highway / Thurmon Tanner / Falcon Parkway</x:v>
       </x:c>
       <x:c r="B9" s="37" t="str">
-        <x:v>Oakwood/Gainesville phases, sewer/DOT agreements, later permits</x:v>
+        <x:v>M-2 quarry/heavy industrial when the buyer wants ordinary logistics</x:v>
       </x:c>
       <x:c r="C9" s="37" t="str">
-        <x:v>Flowery Branch A-to-M-1 ordinances are verified; full multi-city chain is not.</x:v>
+        <x:v>Lead with M-1, road network, utilities, and building geometry.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="56" customHeight="1">
       <x:c r="A10" s="37" t="str">
-        <x:v>Exit 12 / Hines</x:v>
+        <x:v>HB/commercial frontage that can convert to M-1 at Exit 12/14</x:v>
       </x:c>
       <x:c r="B10" s="37" t="str">
-        <x:v>Parcel-to-building crosswalk and permit/CO files</x:v>
+        <x:v>Projects outside or unclear to Flowery Branch city limits</x:v>
       </x:c>
       <x:c r="C10" s="37" t="str">
-        <x:v>Official HB-to-M-1 record is now tied to parcel 08097 000008 and Ordinance 652.</x:v>
+        <x:v>Keep the city-limit analysis tight; do not borrow Oakwood/Hall approvals as city comps.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="56" customHeight="1">
       <x:c r="A11" s="37" t="str">
-        <x:v>Vulcan</x:v>
+        <x:v>A-to-M-1 inside an existing industrial corridor with a utility plan</x:v>
       </x:c>
       <x:c r="B11" s="37" t="str">
-        <x:v>Current operating/permit status</x:v>
+        <x:v>Residential/non-industrial character areas without industrial fabric</x:v>
       </x:c>
       <x:c r="C11" s="37" t="str">
-        <x:v>Final M-2/CUP approval and conditions are verified, but it is heavy industrial rather than logistics.</x:v>
+        <x:v>Agricultural conversion is an infrastructure thesis, not just a rezoning thesis.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="56" customHeight="1">
       <x:c r="A12" s="37" t="str">
-        <x:v>4272 Thurmon Tanner and 4627 Atlanta Highway</x:v>
+        <x:v>M-1 with variance relief for smaller office/warehouse infill</x:v>
       </x:c>
       <x:c r="B12" s="37" t="str">
-        <x:v>Later operational/construction status</x:v>
+        <x:v>Marketed projects with no matched city approval path</x:v>
       </x:c>
       <x:c r="C12" s="37" t="str">
-        <x:v>Useful current City process comps for M-1/CUP and M-1 variance relief.</x:v>
+        <x:v>Use market projects as demand evidence, not entitlement proof.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="56" customHeight="1">
       <x:c r="A13" s="37" t="str">
-        <x:v>Pattillo and Alliance</x:v>
+        <x:v>Project Falcon, Exit 12/Hines, 4627 Atlanta Highway, 4272 Thurmon Tanner</x:v>
       </x:c>
       <x:c r="B13" s="37" t="str">
-        <x:v>Full entitlement/source file</x:v>
+        <x:v>Vulcan and Alliance/Pattillo for different reasons</x:v>
       </x:c>
       <x:c r="C13" s="37" t="str">
-        <x:v>Market signals are useful, but should not be treated as final local approvals.</x:v>
+        <x:v>Color-code conversion risk before pricing land control.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -626,10 +627,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B21" s="37" t="str">
-        <x:v>Respect the ORR boundary</x:v>
+        <x:v>Verify permit posture before closing</x:v>
       </x:c>
       <x:c r="C21" s="37" t="str">
-        <x:v>Public packet review cannot replace permit/CO copies where the county requires open-record requests.</x:v>
+        <x:v>Building permits, COs, utility letters, and site-plan details should be confirmed for the specific parcel before customer reliance.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1413,890 +1414,268 @@
     <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="41" t="str">
-        <x:v>Name</x:v>
+        <x:v>conversion_rating</x:v>
       </x:c>
       <x:c r="B1" s="41" t="str">
-        <x:v>Role</x:v>
+        <x:v>starting_zoning_or_status</x:v>
       </x:c>
       <x:c r="C1" s="41" t="str">
-        <x:v>Organization</x:v>
+        <x:v>starting_character_area_or_context</x:v>
       </x:c>
       <x:c r="D1" s="41" t="str">
-        <x:v>Jurisdiction or case</x:v>
+        <x:v>target_zoning_or_use</x:v>
       </x:c>
       <x:c r="E1" s="41" t="str">
-        <x:v>Player type</x:v>
+        <x:v>customer_read</x:v>
       </x:c>
       <x:c r="F1" s="41" t="str">
-        <x:v>Evidence-based signal</x:v>
+        <x:v>case_examples</x:v>
       </x:c>
       <x:c r="G1" s="41" t="str">
-        <x:v>Confidence</x:v>
+        <x:v>conditions_or_friction</x:v>
       </x:c>
       <x:c r="H1" s="41" t="str">
-        <x:v>Source</x:v>
+        <x:v>acquisition_rule</x:v>
+      </x:c>
+      <x:c r="I1" s="41" t="str">
+        <x:v>primary_source_ids</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="37" t="str">
-        <x:v>Oliver McClellan</x:v>
+        <x:v>Green</x:v>
       </x:c>
       <x:c r="B2" s="37" t="str">
-        <x:v>Mayor</x:v>
+        <x:v>Existing City M-1 industrial zoning</x:v>
       </x:c>
       <x:c r="C2" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>Industrial Employment or established Atlanta Highway / Thurmon Tanner / Falcon Parkway industrial corridor</x:v>
       </x:c>
       <x:c r="D2" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>Office warehouse light manufacturing warehouse variance or site-plan execution</x:v>
       </x:c>
       <x:c r="E2" s="37" t="str">
-        <x:v>Current decision-maker</x:v>
+        <x:v>Best customer starting point inside city limits because the question is usually site constraints not whether industrial belongs there</x:v>
       </x:c>
       <x:c r="F2" s="37" t="str">
-        <x:v>Current mayor listed with 2026 City Council records</x:v>
+        <x:v>4627 Atlanta Highway Business Park existing M-1 with office/warehouse variance</x:v>
       </x:c>
       <x:c r="G2" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Stream buffer impervious setback parking stormwater and construction permits still control execution</x:v>
       </x:c>
       <x:c r="H2" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+        <x:v>Prioritize M-1 sites where building scale access and utilities already match the target product</x:v>
+      </x:c>
+      <x:c r="I2" s="37" t="str">
+        <x:v>S01;S13;S14</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="37" t="str">
-        <x:v>Chris Mundy</x:v>
+        <x:v>Green</x:v>
       </x:c>
       <x:c r="B3" s="37" t="str">
-        <x:v>Councilmember</x:v>
+        <x:v>Highway Business or commercial frontage already planned for industrial-employment transition</x:v>
       </x:c>
       <x:c r="C3" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>Industrial Employment / I-985 interchange logistics context</x:v>
       </x:c>
       <x:c r="D3" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>M-1 warehouse logistics or office-warehouse</x:v>
       </x:c>
       <x:c r="E3" s="37" t="str">
-        <x:v>Current decision-maker</x:v>
+        <x:v>Strong conversion lane when frontage is at Exit 12/14 or Thurmon Tanner and the city can keep commercial frontage where appropriate</x:v>
       </x:c>
       <x:c r="F3" s="37" t="str">
-        <x:v>Current council roster; voted yes on Vulcan first reading in 2021</x:v>
+        <x:v>Exit 12 / Hines HB-to-M-1; Thurmon Tanner Logistics</x:v>
       </x:c>
       <x:c r="G3" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Traffic contribution development agreement buffers detention residential interface and parcel-to-building phasing</x:v>
       </x:c>
       <x:c r="H3" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+        <x:v>Commercial frontage can become industrial when the city can preserve road function and buffer neighbors</x:v>
+      </x:c>
+      <x:c r="I3" s="37" t="str">
+        <x:v>S01;S11</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="37" t="str">
-        <x:v>Joseph Mezzanotte</x:v>
+        <x:v>Yellow</x:v>
       </x:c>
       <x:c r="B4" s="37" t="str">
-        <x:v>Councilmember</x:v>
+        <x:v>Agricultural land inside the city or annexed into a proven industrial corridor</x:v>
       </x:c>
       <x:c r="C4" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>Activity Center or Industrial Employment context with major infrastructure story</x:v>
       </x:c>
       <x:c r="D4" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>M-1 industrial park warehouse or office-warehouse</x:v>
       </x:c>
       <x:c r="E4" s="37" t="str">
-        <x:v>Current decision-maker</x:v>
+        <x:v>Convertible when the project expands an existing industrial corridor and solves sewer road and cross-jurisdiction infrastructure</x:v>
       </x:c>
       <x:c r="F4" s="37" t="str">
-        <x:v>Current council roster</x:v>
+        <x:v>Project Falcon A-to-M-1 Flowery Branch portion</x:v>
       </x:c>
       <x:c r="G4" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Large sewer/pump-station DOT utility easement and multi-jurisdiction coordination can be more important than zoning label</x:v>
       </x:c>
       <x:c r="H4" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+        <x:v>Good land-control candidate only if the infrastructure plan is real and sponsor can carry timing risk</x:v>
+      </x:c>
+      <x:c r="I4" s="37" t="str">
+        <x:v>S08;S09;S10;S22</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="37" t="str">
-        <x:v>Charles Vanderbilt</x:v>
+        <x:v>Yellow</x:v>
       </x:c>
       <x:c r="B5" s="37" t="str">
-        <x:v>Councilmember</x:v>
+        <x:v>Hall County Light Industrial or similar industrial edge annexed into the city</x:v>
       </x:c>
       <x:c r="C5" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>City industrial corridor context but not necessarily freight/logistics use</x:v>
       </x:c>
       <x:c r="D5" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>City M-1 plus CUP or conditions</x:v>
       </x:c>
       <x:c r="E5" s="37" t="str">
-        <x:v>Current decision-maker</x:v>
+        <x:v>Good procedural comp for annexation and M-1 mechanics but not automatically a warehouse/truck precedent</x:v>
       </x:c>
       <x:c r="F5" s="37" t="str">
-        <x:v>Current council roster</x:v>
+        <x:v>4272 Thurmon Tanner Hall County Light Industrial to City M-1 plus CUP</x:v>
       </x:c>
       <x:c r="G5" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Use-specific conditions may limit transferability to freight industrial; later operating status still matters</x:v>
       </x:c>
       <x:c r="H5" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+        <x:v>Use as annexation/M-1 process evidence and separately test freight/logistics fit</x:v>
+      </x:c>
+      <x:c r="I5" s="37" t="str">
+        <x:v>S13;S14</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="37" t="str">
-        <x:v>Pete Lena</x:v>
+        <x:v>Orange</x:v>
       </x:c>
       <x:c r="B6" s="37" t="str">
-        <x:v>Councilmember</x:v>
+        <x:v>Hall County agricultural or rural district annexed to City M-2</x:v>
       </x:c>
       <x:c r="C6" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>Industrial Employment may support heavy industry but neighborhood and environmental fit are decisive</x:v>
       </x:c>
       <x:c r="D6" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>M-2 quarry heavy manufacturing extractive or nuisance-potential industrial use</x:v>
       </x:c>
       <x:c r="E6" s="37" t="str">
-        <x:v>Current decision-maker</x:v>
+        <x:v>Possible but high-scrutiny and not comparable to ordinary warehouse/logistics</x:v>
       </x:c>
       <x:c r="F6" s="37" t="str">
-        <x:v>Current council roster</x:v>
+        <x:v>In-town Vulcan Lands AR III to M-2 plus CUP quarry approval</x:v>
       </x:c>
       <x:c r="G6" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>State permits blasting truck traffic creek/tree impacts berms screening and neighborhood response drive feasibility</x:v>
       </x:c>
       <x:c r="H6" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+        <x:v>Underwrite as a special heavy-industrial thesis with longer schedule and higher community-risk budget</x:v>
+      </x:c>
+      <x:c r="I6" s="37" t="str">
+        <x:v>S12</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="37" t="str">
-        <x:v>William McDaniel</x:v>
+        <x:v>Orange</x:v>
       </x:c>
       <x:c r="B7" s="37" t="str">
-        <x:v>Councilmember</x:v>
+        <x:v>Existing M-1 site needing material relief from buffers setbacks or site constraints</x:v>
       </x:c>
       <x:c r="C7" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>Industrial corridor but physically constrained parcel</x:v>
       </x:c>
       <x:c r="D7" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>Office warehouse or light industrial with variance relief</x:v>
       </x:c>
       <x:c r="E7" s="37" t="str">
-        <x:v>Current decision-maker</x:v>
+        <x:v>Viable for smaller flex/office-warehouse product when the city can condition relief</x:v>
       </x:c>
       <x:c r="F7" s="37" t="str">
-        <x:v>Current council roster</x:v>
+        <x:v>4627 Atlanta Highway stream-buffer and impervious-setback variances</x:v>
       </x:c>
       <x:c r="G7" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Variance risk is lower than full rezoning but construction permits and stormwater still matter</x:v>
       </x:c>
       <x:c r="H7" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+        <x:v>Good infill strategy if the customer can live with smaller buildings and constrained site design</x:v>
+      </x:c>
+      <x:c r="I7" s="37" t="str">
+        <x:v>S13;S14</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="37" t="str">
-        <x:v>Tonya Parrish</x:v>
+        <x:v>Red</x:v>
       </x:c>
       <x:c r="B8" s="37" t="str">
-        <x:v>City Manager</x:v>
+        <x:v>Marketed or under-construction industrial project without a confirmed Flowery Branch city-limit entitlement chain</x:v>
       </x:c>
       <x:c r="C8" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>Potentially Hall/Oakwood/Flowery edge but city jurisdiction not established</x:v>
       </x:c>
       <x:c r="D8" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>Do not rely on as Flowery Branch conversion precedent</x:v>
       </x:c>
       <x:c r="E8" s="37" t="str">
-        <x:v>Senior staff</x:v>
+        <x:v>Useful as I-985 market demand evidence but not as a city-limit zoning template</x:v>
       </x:c>
       <x:c r="F8" s="37" t="str">
-        <x:v>Chief administrative staff listed in current City records</x:v>
+        <x:v>Alliance 985; Pattillo as market/status comp where historic city zoning chain is incomplete</x:v>
       </x:c>
       <x:c r="G8" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Jurisdiction parcel chain permit route and city/county authority must be confirmed before using as comp</x:v>
       </x:c>
       <x:c r="H8" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+        <x:v>Treat as market support only until the exact city-limit approval path is matched</x:v>
+      </x:c>
+      <x:c r="I8" s="37" t="str">
+        <x:v>S20;S21;S23;S25</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="37" t="str">
-        <x:v>Chris McCrary</x:v>
+        <x:v>Red</x:v>
       </x:c>
       <x:c r="B9" s="37" t="str">
-        <x:v>Planning and Community Development Director</x:v>
+        <x:v>Residential neighborhood commercial downtown mixed-use or non-industrial civic character context</x:v>
       </x:c>
       <x:c r="C9" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
+        <x:v>Non-industrial character area or corridor without industrial fabric</x:v>
       </x:c>
       <x:c r="D9" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
+        <x:v>M-1 M-2 or freight-intensive use</x:v>
       </x:c>
       <x:c r="E9" s="37" t="str">
-        <x:v>Staff gatekeeper</x:v>
+        <x:v>Weak customer target inside Flowery Branch city limits because the city code ties M-1/M-2 to Industrial Employment and road-network fit</x:v>
       </x:c>
       <x:c r="F9" s="37" t="str">
-        <x:v>Planning director listed in current City records</x:v>
+        <x:v>No positive city-limit warehouse conversion comp in the reviewed cases</x:v>
       </x:c>
       <x:c r="G9" s="37" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Plan mismatch neighborhood interface local-road truck impacts and political friction dominate</x:v>
       </x:c>
       <x:c r="H9" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="37" t="str">
-        <x:v>Ted Baggett</x:v>
-      </x:c>
-      <x:c r="B10" s="37" t="str">
-        <x:v>City Attorney</x:v>
-      </x:c>
-      <x:c r="C10" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
-      </x:c>
-      <x:c r="D10" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
-      </x:c>
-      <x:c r="E10" s="37" t="str">
-        <x:v>Public counsel</x:v>
-      </x:c>
-      <x:c r="F10" s="37" t="str">
-        <x:v>City attorney listed in current City records</x:v>
-      </x:c>
-      <x:c r="G10" s="37" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="H10" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="37" t="str">
-        <x:v>Peter Woerner</x:v>
-      </x:c>
-      <x:c r="B11" s="37" t="str">
-        <x:v>Public Utilities Director</x:v>
-      </x:c>
-      <x:c r="C11" s="37" t="str">
-        <x:v>City of Flowery Branch</x:v>
-      </x:c>
-      <x:c r="D11" s="37" t="str">
-        <x:v>Flowery Branch</x:v>
-      </x:c>
-      <x:c r="E11" s="37" t="str">
-        <x:v>Utility stakeholder</x:v>
-      </x:c>
-      <x:c r="F11" s="37" t="str">
-        <x:v>Public utilities director listed in current City records</x:v>
-      </x:c>
-      <x:c r="G11" s="37" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="H11" s="37" t="str">
-        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="37" t="str">
-        <x:v>David Gibbs</x:v>
-      </x:c>
-      <x:c r="B12" s="37" t="str">
-        <x:v>Commission Chairman</x:v>
-      </x:c>
-      <x:c r="C12" s="37" t="str">
-        <x:v>Hall County Board of Commissioners</x:v>
-      </x:c>
-      <x:c r="D12" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="E12" s="37" t="str">
-        <x:v>County decision-maker</x:v>
-      </x:c>
-      <x:c r="F12" s="37" t="str">
-        <x:v>Current board chairman</x:v>
-      </x:c>
-      <x:c r="G12" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H12" s="37" t="str">
-        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="37" t="str">
-        <x:v>Kathy Cooper</x:v>
-      </x:c>
-      <x:c r="B13" s="37" t="str">
-        <x:v>District 1 Commissioner</x:v>
-      </x:c>
-      <x:c r="C13" s="37" t="str">
-        <x:v>Hall County Board of Commissioners</x:v>
-      </x:c>
-      <x:c r="D13" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="E13" s="37" t="str">
-        <x:v>County decision-maker</x:v>
-      </x:c>
-      <x:c r="F13" s="37" t="str">
-        <x:v>Current board roster</x:v>
-      </x:c>
-      <x:c r="G13" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H13" s="37" t="str">
-        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="37" t="str">
-        <x:v>Billy Powell</x:v>
-      </x:c>
-      <x:c r="B14" s="37" t="str">
-        <x:v>District 2 Commissioner</x:v>
-      </x:c>
-      <x:c r="C14" s="37" t="str">
-        <x:v>Hall County Board of Commissioners</x:v>
-      </x:c>
-      <x:c r="D14" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="E14" s="37" t="str">
-        <x:v>County decision-maker</x:v>
-      </x:c>
-      <x:c r="F14" s="37" t="str">
-        <x:v>Current board roster</x:v>
-      </x:c>
-      <x:c r="G14" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H14" s="37" t="str">
-        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="37" t="str">
-        <x:v>Gregg Poole</x:v>
-      </x:c>
-      <x:c r="B15" s="37" t="str">
-        <x:v>District 3 Commissioner</x:v>
-      </x:c>
-      <x:c r="C15" s="37" t="str">
-        <x:v>Hall County Board of Commissioners</x:v>
-      </x:c>
-      <x:c r="D15" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="E15" s="37" t="str">
-        <x:v>County decision-maker</x:v>
-      </x:c>
-      <x:c r="F15" s="37" t="str">
-        <x:v>Current board roster</x:v>
-      </x:c>
-      <x:c r="G15" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H15" s="37" t="str">
-        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="37" t="str">
-        <x:v>Jeff Stowe</x:v>
-      </x:c>
-      <x:c r="B16" s="37" t="str">
-        <x:v>District 4 Commissioner</x:v>
-      </x:c>
-      <x:c r="C16" s="37" t="str">
-        <x:v>Hall County Board of Commissioners</x:v>
-      </x:c>
-      <x:c r="D16" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="E16" s="37" t="str">
-        <x:v>County decision-maker</x:v>
-      </x:c>
-      <x:c r="F16" s="37" t="str">
-        <x:v>Current board roster</x:v>
-      </x:c>
-      <x:c r="G16" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H16" s="37" t="str">
-        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="37" t="str">
-        <x:v>Katie Greenway Ahmed</x:v>
-      </x:c>
-      <x:c r="B17" s="37" t="str">
-        <x:v>Director of Planning and Zoning</x:v>
-      </x:c>
-      <x:c r="C17" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="D17" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="E17" s="37" t="str">
-        <x:v>County staff gatekeeper</x:v>
-      </x:c>
-      <x:c r="F17" s="37" t="str">
-        <x:v>Named director March 2026 after serving as Planning and Zoning Administrator</x:v>
-      </x:c>
-      <x:c r="G17" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H17" s="37" t="str">
-        <x:v>https://www.hallcounty.org/m/newsflash/home/detail/1484</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="37" t="str">
-        <x:v>Kristie Turner</x:v>
-      </x:c>
-      <x:c r="B18" s="37" t="str">
-        <x:v>Director of Development Services</x:v>
-      </x:c>
-      <x:c r="C18" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="D18" s="37" t="str">
-        <x:v>Hall County</x:v>
-      </x:c>
-      <x:c r="E18" s="37" t="str">
-        <x:v>County staff gatekeeper</x:v>
-      </x:c>
-      <x:c r="F18" s="37" t="str">
-        <x:v>Named director effective May 2025</x:v>
-      </x:c>
-      <x:c r="G18" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H18" s="37" t="str">
-        <x:v>https://www.hallcounty.org/m/newsflash/home/detail/1392</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Hines</x:v>
-      </x:c>
-      <x:c r="B19" s="37" t="str">
-        <x:v>Developer</x:v>
-      </x:c>
-      <x:c r="C19" s="37" t="str">
-        <x:v>Hines</x:v>
-      </x:c>
-      <x:c r="D19" s="37" t="str">
-        <x:v>Thurmon Tanner Logistics</x:v>
-      </x:c>
-      <x:c r="E19" s="37" t="str">
-        <x:v>Developer</x:v>
-      </x:c>
-      <x:c r="F19" s="37" t="str">
-        <x:v>Started construction on three-building more-than-825k-SF project</x:v>
-      </x:c>
-      <x:c r="G19" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H19" s="37" t="str">
-        <x:v>https://www.hines.com/news/hines-starts-construction-on-thurmon-tanner-logistics</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="37" t="str">
-        <x:v>Ryan Wood</x:v>
-      </x:c>
-      <x:c r="B20" s="37" t="str">
-        <x:v>Managing Director</x:v>
-      </x:c>
-      <x:c r="C20" s="37" t="str">
-        <x:v>Hines</x:v>
-      </x:c>
-      <x:c r="D20" s="37" t="str">
-        <x:v>Thurmon Tanner Logistics</x:v>
-      </x:c>
-      <x:c r="E20" s="37" t="str">
-        <x:v>Developer representative</x:v>
-      </x:c>
-      <x:c r="F20" s="37" t="str">
-        <x:v>Quoted Hines project lead</x:v>
-      </x:c>
-      <x:c r="G20" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H20" s="37" t="str">
-        <x:v>https://www.hines.com/news/hines-starts-construction-on-thurmon-tanner-logistics</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="37" t="str">
-        <x:v>Alliance Industrial Co</x:v>
-      </x:c>
-      <x:c r="B21" s="37" t="str">
-        <x:v>Developer</x:v>
-      </x:c>
-      <x:c r="C21" s="37" t="str">
-        <x:v>Alliance Industrial Co</x:v>
-      </x:c>
-      <x:c r="D21" s="37" t="str">
-        <x:v>Alliance 985 Business Park</x:v>
-      </x:c>
-      <x:c r="E21" s="37" t="str">
-        <x:v>Developer</x:v>
-      </x:c>
-      <x:c r="F21" s="37" t="str">
-        <x:v>Acquired 66.8-acre I-985 site and announced two-building spec development</x:v>
-      </x:c>
-      <x:c r="G21" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H21" s="37" t="str">
-        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="37" t="str">
-        <x:v>Chris Hoag</x:v>
-      </x:c>
-      <x:c r="B22" s="37" t="str">
-        <x:v>Industrial broker</x:v>
-      </x:c>
-      <x:c r="C22" s="37" t="str">
-        <x:v>Avison Young</x:v>
-      </x:c>
-      <x:c r="D22" s="37" t="str">
-        <x:v>Alliance 985 Business Park</x:v>
-      </x:c>
-      <x:c r="E22" s="37" t="str">
-        <x:v>Broker</x:v>
-      </x:c>
-      <x:c r="F22" s="37" t="str">
-        <x:v>Buyer representation team</x:v>
-      </x:c>
-      <x:c r="G22" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H22" s="37" t="str">
-        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="37" t="str">
-        <x:v>Jason Holland</x:v>
-      </x:c>
-      <x:c r="B23" s="37" t="str">
-        <x:v>Industrial broker</x:v>
-      </x:c>
-      <x:c r="C23" s="37" t="str">
-        <x:v>Avison Young</x:v>
-      </x:c>
-      <x:c r="D23" s="37" t="str">
-        <x:v>Alliance 985 Business Park</x:v>
-      </x:c>
-      <x:c r="E23" s="37" t="str">
-        <x:v>Broker</x:v>
-      </x:c>
-      <x:c r="F23" s="37" t="str">
-        <x:v>Buyer representation team</x:v>
-      </x:c>
-      <x:c r="G23" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H23" s="37" t="str">
-        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="37" t="str">
-        <x:v>Andrew Joyner</x:v>
-      </x:c>
-      <x:c r="B24" s="37" t="str">
-        <x:v>Industrial broker</x:v>
-      </x:c>
-      <x:c r="C24" s="37" t="str">
-        <x:v>Avison Young</x:v>
-      </x:c>
-      <x:c r="D24" s="37" t="str">
-        <x:v>Alliance 985 Business Park</x:v>
-      </x:c>
-      <x:c r="E24" s="37" t="str">
-        <x:v>Broker</x:v>
-      </x:c>
-      <x:c r="F24" s="37" t="str">
-        <x:v>Buyer representation team</x:v>
-      </x:c>
-      <x:c r="G24" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H24" s="37" t="str">
-        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="37" t="str">
-        <x:v>Stephen Lovett</x:v>
-      </x:c>
-      <x:c r="B25" s="37" t="str">
-        <x:v>Broker</x:v>
-      </x:c>
-      <x:c r="C25" s="37" t="str">
-        <x:v>Norton Commercial</x:v>
-      </x:c>
-      <x:c r="D25" s="37" t="str">
-        <x:v>Alliance 985 Business Park</x:v>
-      </x:c>
-      <x:c r="E25" s="37" t="str">
-        <x:v>Broker</x:v>
-      </x:c>
-      <x:c r="F25" s="37" t="str">
-        <x:v>Seller representation on a parcel</x:v>
-      </x:c>
-      <x:c r="G25" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H25" s="37" t="str">
-        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="37" t="str">
-        <x:v>Zach Tibbs</x:v>
-      </x:c>
-      <x:c r="B26" s="37" t="str">
-        <x:v>Broker</x:v>
-      </x:c>
-      <x:c r="C26" s="37" t="str">
-        <x:v>Norton Commercial</x:v>
-      </x:c>
-      <x:c r="D26" s="37" t="str">
-        <x:v>Alliance 985 Business Park</x:v>
-      </x:c>
-      <x:c r="E26" s="37" t="str">
-        <x:v>Broker</x:v>
-      </x:c>
-      <x:c r="F26" s="37" t="str">
-        <x:v>Seller representation on a parcel</x:v>
-      </x:c>
-      <x:c r="G26" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H26" s="37" t="str">
-        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="37" t="str">
-        <x:v>CA Ventures</x:v>
-      </x:c>
-      <x:c r="B27" s="37" t="str">
-        <x:v>Developer client</x:v>
-      </x:c>
-      <x:c r="C27" s="37" t="str">
-        <x:v>CA Ventures</x:v>
-      </x:c>
-      <x:c r="D27" s="37" t="str">
-        <x:v>Project Falcon</x:v>
-      </x:c>
-      <x:c r="E27" s="37" t="str">
-        <x:v>Developer</x:v>
-      </x:c>
-      <x:c r="F27" s="37" t="str">
-        <x:v>Named client for two-phase industrial project</x:v>
-      </x:c>
-      <x:c r="G27" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H27" s="37" t="str">
-        <x:v>https://www.reevesyoung.com/case-study/project-falcon/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="37" t="str">
-        <x:v>Reeves + Young</x:v>
-      </x:c>
-      <x:c r="B28" s="37" t="str">
-        <x:v>General contractor</x:v>
-      </x:c>
-      <x:c r="C28" s="37" t="str">
-        <x:v>Reeves + Young</x:v>
-      </x:c>
-      <x:c r="D28" s="37" t="str">
-        <x:v>Project Falcon</x:v>
-      </x:c>
-      <x:c r="E28" s="37" t="str">
-        <x:v>General contractor</x:v>
-      </x:c>
-      <x:c r="F28" s="37" t="str">
-        <x:v>Delivered five-building industrial case study and complex sewer infrastructure</x:v>
-      </x:c>
-      <x:c r="G28" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H28" s="37" t="str">
-        <x:v>https://www.reevesyoung.com/case-study/project-falcon/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="37" t="str">
-        <x:v>Pattillo Industrial Real Estate</x:v>
-      </x:c>
-      <x:c r="B29" s="37" t="str">
-        <x:v>Developer</x:v>
-      </x:c>
-      <x:c r="C29" s="37" t="str">
-        <x:v>Pattillo</x:v>
-      </x:c>
-      <x:c r="D29" s="37" t="str">
-        <x:v>Flowery Branch Business Center</x:v>
-      </x:c>
-      <x:c r="E29" s="37" t="str">
-        <x:v>Developer</x:v>
-      </x:c>
-      <x:c r="F29" s="37" t="str">
-        <x:v>Active BTS land sponsor; Hall County report notes 200k-SF Flowery Branch plan</x:v>
-      </x:c>
-      <x:c r="G29" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H29" s="37" t="str">
-        <x:v>https://www.hallcounty.org/DocumentCenter/View/16821/2025-Annual-Comprehensive-Financial-Report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="37" t="str">
-        <x:v>Ben Stafford</x:v>
-      </x:c>
-      <x:c r="B30" s="37" t="str">
-        <x:v>VP New Investments</x:v>
-      </x:c>
-      <x:c r="C30" s="37" t="str">
-        <x:v>Pattillo Industrial Real Estate</x:v>
-      </x:c>
-      <x:c r="D30" s="37" t="str">
-        <x:v>Flowery Branch Business Center</x:v>
-      </x:c>
-      <x:c r="E30" s="37" t="str">
-        <x:v>Developer representative</x:v>
-      </x:c>
-      <x:c r="F30" s="37" t="str">
-        <x:v>Named in local reporting on grading and project scope</x:v>
-      </x:c>
-      <x:c r="G30" s="37" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="H30" s="37" t="str">
-        <x:v>https://www.yahoo.com/news/whats-grading-off-thurmon-tanner-194800309.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="37" t="str">
-        <x:v>Vulcan Lands Inc.</x:v>
-      </x:c>
-      <x:c r="B31" s="37" t="str">
-        <x:v>Applicant</x:v>
-      </x:c>
-      <x:c r="C31" s="37" t="str">
-        <x:v>Vulcan Lands</x:v>
-      </x:c>
-      <x:c r="D31" s="37" t="str">
-        <x:v>2021 quarry request</x:v>
-      </x:c>
-      <x:c r="E31" s="37" t="str">
-        <x:v>Applicant</x:v>
-      </x:c>
-      <x:c r="F31" s="37" t="str">
-        <x:v>Named annexation/M-2/CUP applicant</x:v>
-      </x:c>
-      <x:c r="G31" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H31" s="37" t="str">
-        <x:v>https://flowerybranchga.granicus.com/DocumentViewer.php?file=flowerybranchga_e40a2aa6-5a5e-4b11-b343-d2cade1fd265.pdf&amp;view=1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="37" t="str">
-        <x:v>Adam Hazell</x:v>
-      </x:c>
-      <x:c r="B32" s="37" t="str">
-        <x:v>DRI contact</x:v>
-      </x:c>
-      <x:c r="C32" s="37" t="str">
-        <x:v>Georgia Mountains Regional Commission</x:v>
-      </x:c>
-      <x:c r="D32" s="37" t="str">
-        <x:v>Regional review</x:v>
-      </x:c>
-      <x:c r="E32" s="37" t="str">
-        <x:v>Regional planning contact</x:v>
-      </x:c>
-      <x:c r="F32" s="37" t="str">
-        <x:v>GMRC DRI program contact</x:v>
-      </x:c>
-      <x:c r="G32" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H32" s="37" t="str">
-        <x:v>https://www.gmrc.ga.gov/dri</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="37" t="str">
-        <x:v>Nikki Chandler</x:v>
-      </x:c>
-      <x:c r="B33" s="37" t="str">
-        <x:v>VP Existing Industry</x:v>
-      </x:c>
-      <x:c r="C33" s="37" t="str">
-        <x:v>Greater Hall Chamber</x:v>
-      </x:c>
-      <x:c r="D33" s="37" t="str">
-        <x:v>Countywide</x:v>
-      </x:c>
-      <x:c r="E33" s="37" t="str">
-        <x:v>Market and economic-development stakeholder</x:v>
-      </x:c>
-      <x:c r="F33" s="37" t="str">
-        <x:v>Existing-industry program contact</x:v>
-      </x:c>
-      <x:c r="G33" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H33" s="37" t="str">
-        <x:v>https://www.ghcc.com/economic-development/existing-industry-program/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="37" t="str">
-        <x:v>Gainesville-Hall County Development Authority</x:v>
-      </x:c>
-      <x:c r="B34" s="37" t="str">
-        <x:v>Industrial incentive authority</x:v>
-      </x:c>
-      <x:c r="C34" s="37" t="str">
-        <x:v>Gainesville-Hall County Development Authority</x:v>
-      </x:c>
-      <x:c r="D34" s="37" t="str">
-        <x:v>Countywide</x:v>
-      </x:c>
-      <x:c r="E34" s="37" t="str">
-        <x:v>Incentive stakeholder</x:v>
-      </x:c>
-      <x:c r="F34" s="37" t="str">
-        <x:v>Can use Investment Assistance Program for qualifying industrial projects</x:v>
-      </x:c>
-      <x:c r="G34" s="37" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H34" s="37" t="str">
-        <x:v>https://www.hallcounty.org/DocumentCenter/View/16821/2025-Annual-Comprehensive-Financial-Report</x:v>
+        <x:v>Avoid unless a specific comprehensive-plan change and infrastructure package are already in motion</x:v>
+      </x:c>
+      <x:c r="I9" s="37" t="str">
+        <x:v>S01;S02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2314,6 +1693,909 @@
     <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="41" t="str">
+        <x:v>Name</x:v>
+      </x:c>
+      <x:c r="B1" s="41" t="str">
+        <x:v>Role</x:v>
+      </x:c>
+      <x:c r="C1" s="41" t="str">
+        <x:v>Organization</x:v>
+      </x:c>
+      <x:c r="D1" s="41" t="str">
+        <x:v>Jurisdiction or case</x:v>
+      </x:c>
+      <x:c r="E1" s="41" t="str">
+        <x:v>Player type</x:v>
+      </x:c>
+      <x:c r="F1" s="41" t="str">
+        <x:v>Evidence-based signal</x:v>
+      </x:c>
+      <x:c r="G1" s="41" t="str">
+        <x:v>Confidence</x:v>
+      </x:c>
+      <x:c r="H1" s="41" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="37" t="str">
+        <x:v>Oliver McClellan</x:v>
+      </x:c>
+      <x:c r="B2" s="37" t="str">
+        <x:v>Mayor</x:v>
+      </x:c>
+      <x:c r="C2" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D2" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E2" s="37" t="str">
+        <x:v>Current decision-maker</x:v>
+      </x:c>
+      <x:c r="F2" s="37" t="str">
+        <x:v>Current mayor listed with 2026 City Council records</x:v>
+      </x:c>
+      <x:c r="G2" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H2" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="37" t="str">
+        <x:v>Chris Mundy</x:v>
+      </x:c>
+      <x:c r="B3" s="37" t="str">
+        <x:v>Councilmember</x:v>
+      </x:c>
+      <x:c r="C3" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D3" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E3" s="37" t="str">
+        <x:v>Current decision-maker</x:v>
+      </x:c>
+      <x:c r="F3" s="37" t="str">
+        <x:v>Current council roster; voted yes on Vulcan first reading in 2021</x:v>
+      </x:c>
+      <x:c r="G3" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H3" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="37" t="str">
+        <x:v>Joseph Mezzanotte</x:v>
+      </x:c>
+      <x:c r="B4" s="37" t="str">
+        <x:v>Councilmember</x:v>
+      </x:c>
+      <x:c r="C4" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D4" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E4" s="37" t="str">
+        <x:v>Current decision-maker</x:v>
+      </x:c>
+      <x:c r="F4" s="37" t="str">
+        <x:v>Current council roster</x:v>
+      </x:c>
+      <x:c r="G4" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H4" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="37" t="str">
+        <x:v>Charles Vanderbilt</x:v>
+      </x:c>
+      <x:c r="B5" s="37" t="str">
+        <x:v>Councilmember</x:v>
+      </x:c>
+      <x:c r="C5" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D5" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E5" s="37" t="str">
+        <x:v>Current decision-maker</x:v>
+      </x:c>
+      <x:c r="F5" s="37" t="str">
+        <x:v>Current council roster</x:v>
+      </x:c>
+      <x:c r="G5" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H5" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="37" t="str">
+        <x:v>Pete Lena</x:v>
+      </x:c>
+      <x:c r="B6" s="37" t="str">
+        <x:v>Councilmember</x:v>
+      </x:c>
+      <x:c r="C6" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D6" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E6" s="37" t="str">
+        <x:v>Current decision-maker</x:v>
+      </x:c>
+      <x:c r="F6" s="37" t="str">
+        <x:v>Current council roster</x:v>
+      </x:c>
+      <x:c r="G6" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H6" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="37" t="str">
+        <x:v>William McDaniel</x:v>
+      </x:c>
+      <x:c r="B7" s="37" t="str">
+        <x:v>Councilmember</x:v>
+      </x:c>
+      <x:c r="C7" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D7" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E7" s="37" t="str">
+        <x:v>Current decision-maker</x:v>
+      </x:c>
+      <x:c r="F7" s="37" t="str">
+        <x:v>Current council roster</x:v>
+      </x:c>
+      <x:c r="G7" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H7" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="37" t="str">
+        <x:v>Tonya Parrish</x:v>
+      </x:c>
+      <x:c r="B8" s="37" t="str">
+        <x:v>City Manager</x:v>
+      </x:c>
+      <x:c r="C8" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D8" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E8" s="37" t="str">
+        <x:v>Senior staff</x:v>
+      </x:c>
+      <x:c r="F8" s="37" t="str">
+        <x:v>Chief administrative staff listed in current City records</x:v>
+      </x:c>
+      <x:c r="G8" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H8" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="37" t="str">
+        <x:v>Chris McCrary</x:v>
+      </x:c>
+      <x:c r="B9" s="37" t="str">
+        <x:v>Planning and Community Development Director</x:v>
+      </x:c>
+      <x:c r="C9" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D9" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E9" s="37" t="str">
+        <x:v>Staff gatekeeper</x:v>
+      </x:c>
+      <x:c r="F9" s="37" t="str">
+        <x:v>Planning director listed in current City records</x:v>
+      </x:c>
+      <x:c r="G9" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H9" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="37" t="str">
+        <x:v>Ted Baggett</x:v>
+      </x:c>
+      <x:c r="B10" s="37" t="str">
+        <x:v>City Attorney</x:v>
+      </x:c>
+      <x:c r="C10" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D10" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E10" s="37" t="str">
+        <x:v>Public counsel</x:v>
+      </x:c>
+      <x:c r="F10" s="37" t="str">
+        <x:v>City attorney listed in current City records</x:v>
+      </x:c>
+      <x:c r="G10" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H10" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="37" t="str">
+        <x:v>Peter Woerner</x:v>
+      </x:c>
+      <x:c r="B11" s="37" t="str">
+        <x:v>Public Utilities Director</x:v>
+      </x:c>
+      <x:c r="C11" s="37" t="str">
+        <x:v>City of Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D11" s="37" t="str">
+        <x:v>Flowery Branch</x:v>
+      </x:c>
+      <x:c r="E11" s="37" t="str">
+        <x:v>Utility stakeholder</x:v>
+      </x:c>
+      <x:c r="F11" s="37" t="str">
+        <x:v>Public utilities director listed in current City records</x:v>
+      </x:c>
+      <x:c r="G11" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H11" s="37" t="str">
+        <x:v>https://mytown.theboringparts.com/city/flowerybranchga/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="37" t="str">
+        <x:v>David Gibbs</x:v>
+      </x:c>
+      <x:c r="B12" s="37" t="str">
+        <x:v>Commission Chairman</x:v>
+      </x:c>
+      <x:c r="C12" s="37" t="str">
+        <x:v>Hall County Board of Commissioners</x:v>
+      </x:c>
+      <x:c r="D12" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="E12" s="37" t="str">
+        <x:v>County decision-maker</x:v>
+      </x:c>
+      <x:c r="F12" s="37" t="str">
+        <x:v>Current board chairman</x:v>
+      </x:c>
+      <x:c r="G12" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H12" s="37" t="str">
+        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="37" t="str">
+        <x:v>Kathy Cooper</x:v>
+      </x:c>
+      <x:c r="B13" s="37" t="str">
+        <x:v>District 1 Commissioner</x:v>
+      </x:c>
+      <x:c r="C13" s="37" t="str">
+        <x:v>Hall County Board of Commissioners</x:v>
+      </x:c>
+      <x:c r="D13" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="E13" s="37" t="str">
+        <x:v>County decision-maker</x:v>
+      </x:c>
+      <x:c r="F13" s="37" t="str">
+        <x:v>Current board roster</x:v>
+      </x:c>
+      <x:c r="G13" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H13" s="37" t="str">
+        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="37" t="str">
+        <x:v>Billy Powell</x:v>
+      </x:c>
+      <x:c r="B14" s="37" t="str">
+        <x:v>District 2 Commissioner</x:v>
+      </x:c>
+      <x:c r="C14" s="37" t="str">
+        <x:v>Hall County Board of Commissioners</x:v>
+      </x:c>
+      <x:c r="D14" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="E14" s="37" t="str">
+        <x:v>County decision-maker</x:v>
+      </x:c>
+      <x:c r="F14" s="37" t="str">
+        <x:v>Current board roster</x:v>
+      </x:c>
+      <x:c r="G14" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H14" s="37" t="str">
+        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="37" t="str">
+        <x:v>Gregg Poole</x:v>
+      </x:c>
+      <x:c r="B15" s="37" t="str">
+        <x:v>District 3 Commissioner</x:v>
+      </x:c>
+      <x:c r="C15" s="37" t="str">
+        <x:v>Hall County Board of Commissioners</x:v>
+      </x:c>
+      <x:c r="D15" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="E15" s="37" t="str">
+        <x:v>County decision-maker</x:v>
+      </x:c>
+      <x:c r="F15" s="37" t="str">
+        <x:v>Current board roster</x:v>
+      </x:c>
+      <x:c r="G15" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H15" s="37" t="str">
+        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="37" t="str">
+        <x:v>Jeff Stowe</x:v>
+      </x:c>
+      <x:c r="B16" s="37" t="str">
+        <x:v>District 4 Commissioner</x:v>
+      </x:c>
+      <x:c r="C16" s="37" t="str">
+        <x:v>Hall County Board of Commissioners</x:v>
+      </x:c>
+      <x:c r="D16" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="E16" s="37" t="str">
+        <x:v>County decision-maker</x:v>
+      </x:c>
+      <x:c r="F16" s="37" t="str">
+        <x:v>Current board roster</x:v>
+      </x:c>
+      <x:c r="G16" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H16" s="37" t="str">
+        <x:v>https://www.hallcounty.org/Directory.aspx?DID=93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="37" t="str">
+        <x:v>Katie Greenway Ahmed</x:v>
+      </x:c>
+      <x:c r="B17" s="37" t="str">
+        <x:v>Director of Planning and Zoning</x:v>
+      </x:c>
+      <x:c r="C17" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="D17" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="E17" s="37" t="str">
+        <x:v>County staff gatekeeper</x:v>
+      </x:c>
+      <x:c r="F17" s="37" t="str">
+        <x:v>Named director March 2026 after serving as Planning and Zoning Administrator</x:v>
+      </x:c>
+      <x:c r="G17" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H17" s="37" t="str">
+        <x:v>https://www.hallcounty.org/m/newsflash/home/detail/1484</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="37" t="str">
+        <x:v>Kristie Turner</x:v>
+      </x:c>
+      <x:c r="B18" s="37" t="str">
+        <x:v>Director of Development Services</x:v>
+      </x:c>
+      <x:c r="C18" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="D18" s="37" t="str">
+        <x:v>Hall County</x:v>
+      </x:c>
+      <x:c r="E18" s="37" t="str">
+        <x:v>County staff gatekeeper</x:v>
+      </x:c>
+      <x:c r="F18" s="37" t="str">
+        <x:v>Named director effective May 2025</x:v>
+      </x:c>
+      <x:c r="G18" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H18" s="37" t="str">
+        <x:v>https://www.hallcounty.org/m/newsflash/home/detail/1392</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="37" t="str">
+        <x:v>Hines</x:v>
+      </x:c>
+      <x:c r="B19" s="37" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="C19" s="37" t="str">
+        <x:v>Hines</x:v>
+      </x:c>
+      <x:c r="D19" s="37" t="str">
+        <x:v>Thurmon Tanner Logistics</x:v>
+      </x:c>
+      <x:c r="E19" s="37" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="F19" s="37" t="str">
+        <x:v>Started construction on three-building more-than-825k-SF project</x:v>
+      </x:c>
+      <x:c r="G19" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H19" s="37" t="str">
+        <x:v>https://www.hines.com/news/hines-starts-construction-on-thurmon-tanner-logistics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="37" t="str">
+        <x:v>Ryan Wood</x:v>
+      </x:c>
+      <x:c r="B20" s="37" t="str">
+        <x:v>Managing Director</x:v>
+      </x:c>
+      <x:c r="C20" s="37" t="str">
+        <x:v>Hines</x:v>
+      </x:c>
+      <x:c r="D20" s="37" t="str">
+        <x:v>Thurmon Tanner Logistics</x:v>
+      </x:c>
+      <x:c r="E20" s="37" t="str">
+        <x:v>Developer representative</x:v>
+      </x:c>
+      <x:c r="F20" s="37" t="str">
+        <x:v>Quoted Hines project lead</x:v>
+      </x:c>
+      <x:c r="G20" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H20" s="37" t="str">
+        <x:v>https://www.hines.com/news/hines-starts-construction-on-thurmon-tanner-logistics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="37" t="str">
+        <x:v>Alliance Industrial Co</x:v>
+      </x:c>
+      <x:c r="B21" s="37" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="C21" s="37" t="str">
+        <x:v>Alliance Industrial Co</x:v>
+      </x:c>
+      <x:c r="D21" s="37" t="str">
+        <x:v>Alliance 985 Business Park</x:v>
+      </x:c>
+      <x:c r="E21" s="37" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="F21" s="37" t="str">
+        <x:v>Acquired 66.8-acre I-985 site and announced two-building spec development</x:v>
+      </x:c>
+      <x:c r="G21" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H21" s="37" t="str">
+        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="37" t="str">
+        <x:v>Chris Hoag</x:v>
+      </x:c>
+      <x:c r="B22" s="37" t="str">
+        <x:v>Industrial broker</x:v>
+      </x:c>
+      <x:c r="C22" s="37" t="str">
+        <x:v>Avison Young</x:v>
+      </x:c>
+      <x:c r="D22" s="37" t="str">
+        <x:v>Alliance 985 Business Park</x:v>
+      </x:c>
+      <x:c r="E22" s="37" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="F22" s="37" t="str">
+        <x:v>Buyer representation team</x:v>
+      </x:c>
+      <x:c r="G22" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H22" s="37" t="str">
+        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="37" t="str">
+        <x:v>Jason Holland</x:v>
+      </x:c>
+      <x:c r="B23" s="37" t="str">
+        <x:v>Industrial broker</x:v>
+      </x:c>
+      <x:c r="C23" s="37" t="str">
+        <x:v>Avison Young</x:v>
+      </x:c>
+      <x:c r="D23" s="37" t="str">
+        <x:v>Alliance 985 Business Park</x:v>
+      </x:c>
+      <x:c r="E23" s="37" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="F23" s="37" t="str">
+        <x:v>Buyer representation team</x:v>
+      </x:c>
+      <x:c r="G23" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H23" s="37" t="str">
+        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="37" t="str">
+        <x:v>Andrew Joyner</x:v>
+      </x:c>
+      <x:c r="B24" s="37" t="str">
+        <x:v>Industrial broker</x:v>
+      </x:c>
+      <x:c r="C24" s="37" t="str">
+        <x:v>Avison Young</x:v>
+      </x:c>
+      <x:c r="D24" s="37" t="str">
+        <x:v>Alliance 985 Business Park</x:v>
+      </x:c>
+      <x:c r="E24" s="37" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="F24" s="37" t="str">
+        <x:v>Buyer representation team</x:v>
+      </x:c>
+      <x:c r="G24" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H24" s="37" t="str">
+        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="37" t="str">
+        <x:v>Stephen Lovett</x:v>
+      </x:c>
+      <x:c r="B25" s="37" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="C25" s="37" t="str">
+        <x:v>Norton Commercial</x:v>
+      </x:c>
+      <x:c r="D25" s="37" t="str">
+        <x:v>Alliance 985 Business Park</x:v>
+      </x:c>
+      <x:c r="E25" s="37" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="F25" s="37" t="str">
+        <x:v>Seller representation on a parcel</x:v>
+      </x:c>
+      <x:c r="G25" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H25" s="37" t="str">
+        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="37" t="str">
+        <x:v>Zach Tibbs</x:v>
+      </x:c>
+      <x:c r="B26" s="37" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="C26" s="37" t="str">
+        <x:v>Norton Commercial</x:v>
+      </x:c>
+      <x:c r="D26" s="37" t="str">
+        <x:v>Alliance 985 Business Park</x:v>
+      </x:c>
+      <x:c r="E26" s="37" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="F26" s="37" t="str">
+        <x:v>Seller representation on a parcel</x:v>
+      </x:c>
+      <x:c r="G26" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H26" s="37" t="str">
+        <x:v>https://rebusinessonline.com/avison-young-arranges-sale-of-66-8-acres-near-new-northeast-georgia-inland-port/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="37" t="str">
+        <x:v>CA Ventures</x:v>
+      </x:c>
+      <x:c r="B27" s="37" t="str">
+        <x:v>Developer client</x:v>
+      </x:c>
+      <x:c r="C27" s="37" t="str">
+        <x:v>CA Ventures</x:v>
+      </x:c>
+      <x:c r="D27" s="37" t="str">
+        <x:v>Project Falcon</x:v>
+      </x:c>
+      <x:c r="E27" s="37" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="F27" s="37" t="str">
+        <x:v>Named client for two-phase industrial project</x:v>
+      </x:c>
+      <x:c r="G27" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H27" s="37" t="str">
+        <x:v>https://www.reevesyoung.com/case-study/project-falcon/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="37" t="str">
+        <x:v>Reeves + Young</x:v>
+      </x:c>
+      <x:c r="B28" s="37" t="str">
+        <x:v>General contractor</x:v>
+      </x:c>
+      <x:c r="C28" s="37" t="str">
+        <x:v>Reeves + Young</x:v>
+      </x:c>
+      <x:c r="D28" s="37" t="str">
+        <x:v>Project Falcon</x:v>
+      </x:c>
+      <x:c r="E28" s="37" t="str">
+        <x:v>General contractor</x:v>
+      </x:c>
+      <x:c r="F28" s="37" t="str">
+        <x:v>Delivered five-building industrial case study and complex sewer infrastructure</x:v>
+      </x:c>
+      <x:c r="G28" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H28" s="37" t="str">
+        <x:v>https://www.reevesyoung.com/case-study/project-falcon/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="37" t="str">
+        <x:v>Pattillo Industrial Real Estate</x:v>
+      </x:c>
+      <x:c r="B29" s="37" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="C29" s="37" t="str">
+        <x:v>Pattillo</x:v>
+      </x:c>
+      <x:c r="D29" s="37" t="str">
+        <x:v>Flowery Branch Business Center</x:v>
+      </x:c>
+      <x:c r="E29" s="37" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="F29" s="37" t="str">
+        <x:v>Active BTS land sponsor; Hall County report notes 200k-SF Flowery Branch plan</x:v>
+      </x:c>
+      <x:c r="G29" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H29" s="37" t="str">
+        <x:v>https://www.hallcounty.org/DocumentCenter/View/16821/2025-Annual-Comprehensive-Financial-Report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="37" t="str">
+        <x:v>Ben Stafford</x:v>
+      </x:c>
+      <x:c r="B30" s="37" t="str">
+        <x:v>VP New Investments</x:v>
+      </x:c>
+      <x:c r="C30" s="37" t="str">
+        <x:v>Pattillo Industrial Real Estate</x:v>
+      </x:c>
+      <x:c r="D30" s="37" t="str">
+        <x:v>Flowery Branch Business Center</x:v>
+      </x:c>
+      <x:c r="E30" s="37" t="str">
+        <x:v>Developer representative</x:v>
+      </x:c>
+      <x:c r="F30" s="37" t="str">
+        <x:v>Named in local reporting on grading and project scope</x:v>
+      </x:c>
+      <x:c r="G30" s="37" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H30" s="37" t="str">
+        <x:v>https://www.yahoo.com/news/whats-grading-off-thurmon-tanner-194800309.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="37" t="str">
+        <x:v>Vulcan Lands Inc.</x:v>
+      </x:c>
+      <x:c r="B31" s="37" t="str">
+        <x:v>Applicant</x:v>
+      </x:c>
+      <x:c r="C31" s="37" t="str">
+        <x:v>Vulcan Lands</x:v>
+      </x:c>
+      <x:c r="D31" s="37" t="str">
+        <x:v>2021 quarry request</x:v>
+      </x:c>
+      <x:c r="E31" s="37" t="str">
+        <x:v>Applicant</x:v>
+      </x:c>
+      <x:c r="F31" s="37" t="str">
+        <x:v>Named annexation/M-2/CUP applicant</x:v>
+      </x:c>
+      <x:c r="G31" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H31" s="37" t="str">
+        <x:v>https://flowerybranchga.granicus.com/DocumentViewer.php?file=flowerybranchga_e40a2aa6-5a5e-4b11-b343-d2cade1fd265.pdf&amp;view=1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="37" t="str">
+        <x:v>Adam Hazell</x:v>
+      </x:c>
+      <x:c r="B32" s="37" t="str">
+        <x:v>DRI contact</x:v>
+      </x:c>
+      <x:c r="C32" s="37" t="str">
+        <x:v>Georgia Mountains Regional Commission</x:v>
+      </x:c>
+      <x:c r="D32" s="37" t="str">
+        <x:v>Regional review</x:v>
+      </x:c>
+      <x:c r="E32" s="37" t="str">
+        <x:v>Regional planning contact</x:v>
+      </x:c>
+      <x:c r="F32" s="37" t="str">
+        <x:v>GMRC DRI program contact</x:v>
+      </x:c>
+      <x:c r="G32" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H32" s="37" t="str">
+        <x:v>https://www.gmrc.ga.gov/dri</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="37" t="str">
+        <x:v>Nikki Chandler</x:v>
+      </x:c>
+      <x:c r="B33" s="37" t="str">
+        <x:v>VP Existing Industry</x:v>
+      </x:c>
+      <x:c r="C33" s="37" t="str">
+        <x:v>Greater Hall Chamber</x:v>
+      </x:c>
+      <x:c r="D33" s="37" t="str">
+        <x:v>Countywide</x:v>
+      </x:c>
+      <x:c r="E33" s="37" t="str">
+        <x:v>Market and economic-development stakeholder</x:v>
+      </x:c>
+      <x:c r="F33" s="37" t="str">
+        <x:v>Existing-industry program contact</x:v>
+      </x:c>
+      <x:c r="G33" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H33" s="37" t="str">
+        <x:v>https://www.ghcc.com/economic-development/existing-industry-program/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="37" t="str">
+        <x:v>Gainesville-Hall County Development Authority</x:v>
+      </x:c>
+      <x:c r="B34" s="37" t="str">
+        <x:v>Industrial incentive authority</x:v>
+      </x:c>
+      <x:c r="C34" s="37" t="str">
+        <x:v>Gainesville-Hall County Development Authority</x:v>
+      </x:c>
+      <x:c r="D34" s="37" t="str">
+        <x:v>Countywide</x:v>
+      </x:c>
+      <x:c r="E34" s="37" t="str">
+        <x:v>Incentive stakeholder</x:v>
+      </x:c>
+      <x:c r="F34" s="37" t="str">
+        <x:v>Can use Investment Assistance Program for qualifying industrial projects</x:v>
+      </x:c>
+      <x:c r="G34" s="37" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H34" s="37" t="str">
+        <x:v>https://www.hallcounty.org/DocumentCenter/View/16821/2025-Annual-Comprehensive-Financial-Report</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2350,7 +2632,7 @@
         <x:v>M-1 and M-2 purpose and use framework</x:v>
       </x:c>
       <x:c r="E2" s="37" t="str">
-        <x:v>Primary legal source current through Ordinance 779 enacted April 2 2026</x:v>
+        <x:v>Primary legal source; live Municode text identifies M-1 and M-2 as implementing Industrial Employment and includes amendments through Ordinance 786 enacted June 4 2026</x:v>
       </x:c>
       <x:c r="F2" s="37" t="str">
         <x:v>https://library.municode.com/ga/flowery_branch/codes/code_of_ordinances?nodeId=APXCZOOR_ART9NOZODI</x:v>

</xml_diff>